<commit_message>
[ add 字段名 execel]
</commit_message>
<xml_diff>
--- a/erp-server/erp-server-plm/src/main/resources/excel/taskTime.xlsx
+++ b/erp-server/erp-server-plm/src/main/resources/excel/taskTime.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t>产品名称</t>
   </si>
@@ -48,6 +48,9 @@
     <t>延期任务数量</t>
   </si>
   <si>
+    <t>产品创建时间</t>
+  </si>
+  <si>
     <t>{.productName}</t>
   </si>
   <si>
@@ -76,6 +79,12 @@
   </si>
   <si>
     <t>{.delayTaskNum}</t>
+  </si>
+  <si>
+    <t>{.productCreateDate}</t>
+  </si>
+  <si>
+    <t>{.productApprovalDate}</t>
   </si>
 </sst>
 </file>
@@ -1061,7 +1070,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="1"/>
   <cols>
     <col min="1" max="1" width="8.5" customWidth="1"/>
@@ -1073,9 +1082,10 @@
     <col min="8" max="8" width="14.125" customWidth="1"/>
     <col min="9" max="9" width="14.75" customWidth="1"/>
     <col min="10" max="10" width="18.5" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1106,37 +1116,49 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:12">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>